<commit_message>
Add archive shape checks and richer fixture query coverage.
Lock the required xlsx sheet/header contract for the e2e fixture and create-template output, and expand the fixture so compose tests cover alternate subjects, levels, slash shorthand, and missing lookups.
</commit_message>
<xml_diff>
--- a/fixtures/minimal_prompt_archive.xlsx
+++ b/fixtures/minimal_prompt_archive.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="36">
   <si>
     <t>Name</t>
   </si>
@@ -38,6 +38,12 @@
     <t>BODY_ALPHA</t>
   </si>
   <si>
+    <t>Beta</t>
+  </si>
+  <si>
+    <t>BODY_BETA</t>
+  </si>
+  <si>
     <t>Level</t>
   </si>
   <si>
@@ -56,22 +62,70 @@
     <t>OUTFIT_1_1</t>
   </si>
   <si>
+    <t>Outfit L5-30</t>
+  </si>
+  <si>
+    <t>OUTFIT_5_30</t>
+  </si>
+  <si>
+    <t>Outfit L2-02</t>
+  </si>
+  <si>
+    <t>OUTFIT_2_2</t>
+  </si>
+  <si>
     <t>Pose L2-01</t>
   </si>
   <si>
     <t>POSE_2_1</t>
   </si>
   <si>
+    <t>Pose L1-01</t>
+  </si>
+  <si>
+    <t>POSE_1_1</t>
+  </si>
+  <si>
+    <t>Pose L3-05</t>
+  </si>
+  <si>
+    <t>POSE_3_5</t>
+  </si>
+  <si>
     <t>Action L1-02</t>
   </si>
   <si>
     <t>ACTION_1_2</t>
   </si>
   <si>
+    <t>Action L4-10</t>
+  </si>
+  <si>
+    <t>ACTION_4_10</t>
+  </si>
+  <si>
+    <t>Action L2-03</t>
+  </si>
+  <si>
+    <t>ACTION_2_3</t>
+  </si>
+  <si>
     <t>Scene L3-01</t>
   </si>
   <si>
     <t>SCENE_3_1</t>
+  </si>
+  <si>
+    <t>Scene L1-01</t>
+  </si>
+  <si>
+    <t>SCENE_1_1</t>
+  </si>
+  <si>
+    <t>Scene L5-15</t>
+  </si>
+  <si>
+    <t>SCENE_5_15</t>
   </si>
 </sst>
 </file>
@@ -403,7 +457,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D2"/>
+  <dimension ref="A1:D3"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:4">
@@ -428,6 +482,14 @@
         <v>5</v>
       </c>
     </row>
+    <row r="3" spans="1:4">
+      <c r="A3" t="s">
+        <v>6</v>
+      </c>
+      <c r="B3" t="s">
+        <v>7</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -435,7 +497,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D2"/>
+  <dimension ref="A1:D4"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:4">
@@ -443,27 +505,55 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="C1" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="D1" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
     </row>
     <row r="2" spans="1:4">
       <c r="A2" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="B2">
         <v>1</v>
       </c>
       <c r="C2" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="D2" t="s">
-        <v>11</v>
+        <v>13</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4">
+      <c r="A3" t="s">
+        <v>14</v>
+      </c>
+      <c r="B3">
+        <v>5</v>
+      </c>
+      <c r="C3" t="s">
+        <v>12</v>
+      </c>
+      <c r="D3" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4">
+      <c r="A4" t="s">
+        <v>16</v>
+      </c>
+      <c r="B4">
+        <v>2</v>
+      </c>
+      <c r="C4" t="s">
+        <v>12</v>
+      </c>
+      <c r="D4" t="s">
+        <v>17</v>
       </c>
     </row>
   </sheetData>
@@ -473,7 +563,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D2"/>
+  <dimension ref="A1:D4"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:4">
@@ -481,27 +571,55 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="C1" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="D1" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
     </row>
     <row r="2" spans="1:4">
       <c r="A2" t="s">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="B2">
         <v>2</v>
       </c>
       <c r="C2" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="D2" t="s">
-        <v>13</v>
+        <v>19</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4">
+      <c r="A3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B3">
+        <v>1</v>
+      </c>
+      <c r="C3" t="s">
+        <v>12</v>
+      </c>
+      <c r="D3" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4">
+      <c r="A4" t="s">
+        <v>22</v>
+      </c>
+      <c r="B4">
+        <v>3</v>
+      </c>
+      <c r="C4" t="s">
+        <v>12</v>
+      </c>
+      <c r="D4" t="s">
+        <v>23</v>
       </c>
     </row>
   </sheetData>
@@ -511,7 +629,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D2"/>
+  <dimension ref="A1:D4"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:4">
@@ -519,27 +637,55 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="C1" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="D1" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
     </row>
     <row r="2" spans="1:4">
       <c r="A2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="B2">
         <v>1</v>
       </c>
       <c r="C2" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="D2" t="s">
-        <v>15</v>
+        <v>25</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4">
+      <c r="A3" t="s">
+        <v>26</v>
+      </c>
+      <c r="B3">
+        <v>4</v>
+      </c>
+      <c r="C3" t="s">
+        <v>12</v>
+      </c>
+      <c r="D3" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4">
+      <c r="A4" t="s">
+        <v>28</v>
+      </c>
+      <c r="B4">
+        <v>2</v>
+      </c>
+      <c r="C4" t="s">
+        <v>12</v>
+      </c>
+      <c r="D4" t="s">
+        <v>29</v>
       </c>
     </row>
   </sheetData>
@@ -549,7 +695,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D2"/>
+  <dimension ref="A1:D4"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:4">
@@ -557,27 +703,55 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="C1" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="D1" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
     </row>
     <row r="2" spans="1:4">
       <c r="A2" t="s">
-        <v>16</v>
+        <v>30</v>
       </c>
       <c r="B2">
         <v>3</v>
       </c>
       <c r="C2" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="D2" t="s">
-        <v>17</v>
+        <v>31</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4">
+      <c r="A3" t="s">
+        <v>32</v>
+      </c>
+      <c r="B3">
+        <v>1</v>
+      </c>
+      <c r="C3" t="s">
+        <v>12</v>
+      </c>
+      <c r="D3" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4">
+      <c r="A4" t="s">
+        <v>34</v>
+      </c>
+      <c r="B4">
+        <v>5</v>
+      </c>
+      <c r="C4" t="s">
+        <v>12</v>
+      </c>
+      <c r="D4" t="s">
+        <v>35</v>
       </c>
     </row>
   </sheetData>

</xml_diff>